<commit_message>
updated backlog, split up in 3 categories
</commit_message>
<xml_diff>
--- a/ProductBacklog.xlsx
+++ b/ProductBacklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\IdeaProjects\TUe-tycoon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C994D45-4242-422A-815E-DE71078228B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F27991-5A07-4E6C-AC14-5FEFBF39FD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A18C0AB4-C4B4-4CEE-A740-ABC1F7C2C92A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
   <si>
     <t>Product Backlog TU/e Tycoon</t>
   </si>
@@ -53,76 +53,170 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Main game window</t>
-  </si>
-  <si>
-    <t>Launch the app; a window shows the knowledge points, ECTS, current quartile, and an empty BSA progress bar. Resize the window and the layout adapts.</t>
-  </si>
-  <si>
-    <t>No absolute positioning</t>
-  </si>
-  <si>
     <t>Study action</t>
   </si>
   <si>
-    <t>Click on the study button and see the knowledge points go up</t>
-  </si>
-  <si>
-    <t>Amount of knowledge points gained based on upgrades</t>
-  </si>
-  <si>
-    <t>Hire students</t>
-  </si>
-  <si>
     <t>Click on the hire student upgrade button; see updated knowledge per second; substract knowledge points as payment</t>
   </si>
   <si>
-    <t>Complete course</t>
-  </si>
-  <si>
-    <t>Select one of the three courses of this quartile; select complete asignment; see ECTS bar go up; see knowledge points go down; gain a knowledge boost for a limited time</t>
-  </si>
-  <si>
-    <t>Save progress</t>
-  </si>
-  <si>
-    <t>Click the save button, close the game; reopen the game; progress should not be lost</t>
-  </si>
-  <si>
     <t>Timer</t>
   </si>
   <si>
-    <t>Play the game and see the timer go down; when the timer reaches zero you see a lost screen</t>
-  </si>
-  <si>
     <t>price changes depending on how many students you already have, can't buy if you don't have enough knowledge</t>
   </si>
   <si>
-    <t>End of game</t>
-  </si>
-  <si>
-    <t>use a savefile in project folder, missing or corrupt file gives error</t>
-  </si>
-  <si>
-    <t>When you do your last rebirth you get a screen showing if you reached your BSA or not</t>
-  </si>
-  <si>
-    <t>&gt;45 credits -&gt; succesfull</t>
-  </si>
-  <si>
     <t>rebirth</t>
   </si>
   <si>
     <t>Click the rebirth button; knowledge and upgrades reset; you get a permanent bonus</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Rendering</t>
+  </si>
+  <si>
+    <t>Mechanics</t>
+  </si>
+  <si>
+    <t>Credit progress</t>
+  </si>
+  <si>
+    <t>Starts at 0, when completing course it goes up</t>
+  </si>
+  <si>
+    <t>maximum  60</t>
+  </si>
+  <si>
+    <t>Knowledge</t>
+  </si>
+  <si>
+    <t>Starts at 0, goes up when you click study, or automatically when upgrades are bought, goes down when buying upgrades or completing courses</t>
+  </si>
+  <si>
+    <t>Knowledge/second (kps)</t>
+  </si>
+  <si>
+    <t>starts at 0, goes up when upgrades are bought</t>
+  </si>
+  <si>
+    <t>resets after rebirth</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>starts at 0, goes up when "hire student" is bought</t>
+  </si>
+  <si>
+    <t>Quartile</t>
+  </si>
+  <si>
+    <t>Starts at 1, goes up when rebirthed</t>
+  </si>
+  <si>
+    <t>maximum 4</t>
+  </si>
+  <si>
+    <t>multiplier</t>
+  </si>
+  <si>
+    <t>increases by 0,2 per rebirth</t>
+  </si>
+  <si>
+    <t>coffee</t>
+  </si>
+  <si>
+    <t>gameplay menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When game is booted, show all buttons and variables </t>
+  </si>
+  <si>
+    <t>save</t>
+  </si>
+  <si>
+    <t>shows confirmation after clicking the save button</t>
+  </si>
+  <si>
+    <t>shows confirmation after clicking the rebirth button</t>
+  </si>
+  <si>
+    <t>BSA report</t>
+  </si>
+  <si>
+    <t>after rebirthing the 4th time or when the timer runs out shows if you achieved your bsa or not</t>
+  </si>
+  <si>
+    <t>Makes knowledge go up</t>
+  </si>
+  <si>
+    <t>hire students</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go to lecture </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click on the "go to lecture" upgrade button; you can't click on the study button for 10 seconds; afterwards knowledge per click goes up; </t>
+  </si>
+  <si>
+    <t>after being bought the time wasted on lecture goes up</t>
+  </si>
+  <si>
+    <t>knowledge/click (kpc)</t>
+  </si>
+  <si>
+    <t>Starts at 1, goes up when go to lecture is bought</t>
+  </si>
+  <si>
+    <t>Starts at 1 hour and ticks down till zero or when the game is finished</t>
+  </si>
+  <si>
+    <t>Saving</t>
+  </si>
+  <si>
+    <t>clicking the save button saves progress to a savefile;</t>
+  </si>
+  <si>
+    <t>add error message for missing save file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exit </t>
+  </si>
+  <si>
+    <t>close the program</t>
+  </si>
+  <si>
+    <t>doesn't save</t>
+  </si>
+  <si>
+    <t>Extras</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -163,9 +257,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -173,6 +267,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -576,111 +676,113 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
+      <c r="B5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
@@ -690,11 +792,13 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>10</v>
       </c>
-      <c r="B14" s="2"/>
+      <c r="B14" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
     </row>
@@ -702,32 +806,48 @@
       <c r="A15" s="2">
         <v>11</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
+      <c r="B15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>12</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="B16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>13</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+      <c r="B17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>14</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
+      <c r="B18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -738,11 +858,13 @@
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>16</v>
       </c>
-      <c r="B20" s="2"/>
+      <c r="B20" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
     </row>
@@ -750,56 +872,92 @@
       <c r="A21" s="2">
         <v>17</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
+      <c r="B21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>18</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="B22" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>19</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="B23" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>20</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+      <c r="B24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>21</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="B25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>22</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>23</v>
       </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="B27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -807,7 +965,7 @@
         <v>24</v>
       </c>
       <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="C28" s="3"/>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -823,31 +981,33 @@
         <v>26</v>
       </c>
       <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>27</v>
       </c>
       <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
+      <c r="C31" s="3"/>
       <c r="D31" s="2"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>28</v>
       </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
+      <c r="B32" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>29</v>
       </c>
       <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
+      <c r="C33" s="3"/>
       <c r="D33" s="2"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -855,7 +1015,7 @@
         <v>30</v>
       </c>
       <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
+      <c r="C34" s="3"/>
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -863,7 +1023,7 @@
         <v>31</v>
       </c>
       <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
+      <c r="C35" s="3"/>
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -878,7 +1038,9 @@
       <c r="A37" s="2">
         <v>33</v>
       </c>
-      <c r="B37" s="2"/>
+      <c r="B37" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
     </row>
@@ -886,10 +1048,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:D3"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated backlog to reflect added changes
</commit_message>
<xml_diff>
--- a/ProductBacklog.xlsx
+++ b/ProductBacklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\IdeaProjects\TUe-tycoon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F27991-5A07-4E6C-AC14-5FEFBF39FD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB69A3F-5359-4D72-B68D-D31F3F180F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A18C0AB4-C4B4-4CEE-A740-ABC1F7C2C92A}"/>
   </bookViews>
@@ -122,9 +122,6 @@
     <t>multiplier</t>
   </si>
   <si>
-    <t>increases by 0,2 per rebirth</t>
-  </si>
-  <si>
     <t>coffee</t>
   </si>
   <si>
@@ -137,12 +134,6 @@
     <t>save</t>
   </si>
   <si>
-    <t>shows confirmation after clicking the save button</t>
-  </si>
-  <si>
-    <t>shows confirmation after clicking the rebirth button</t>
-  </si>
-  <si>
     <t>BSA report</t>
   </si>
   <si>
@@ -179,9 +170,6 @@
     <t>clicking the save button saves progress to a savefile;</t>
   </si>
   <si>
-    <t>add error message for missing save file</t>
-  </si>
-  <si>
     <t xml:space="preserve">exit </t>
   </si>
   <si>
@@ -192,13 +180,25 @@
   </si>
   <si>
     <t>Extras</t>
+  </si>
+  <si>
+    <t>increase is based on a complicated formula based on all current stats</t>
+  </si>
+  <si>
+    <t>when booting the game up again, see that all variables were saved</t>
+  </si>
+  <si>
+    <t>see that the multiplier went up and that the other variables were reset</t>
+  </si>
+  <si>
+    <t>when save file is missing, create one</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -236,6 +236,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -257,11 +265,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -273,6 +278,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -308,10 +322,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6C1DFACB-6490-4682-AD2B-D709FCE2013B}" name="Table1" displayName="Table1" ref="A4:D37" totalsRowShown="0">
   <autoFilter ref="A4:D37" xr:uid="{6C1DFACB-6490-4682-AD2B-D709FCE2013B}"/>
   <tableColumns count="4">
-    <tableColumn id="7" xr3:uid="{45651187-7C4C-426E-8BC7-943CD802C12A}" name="#" dataDxfId="0"/>
-    <tableColumn id="1" xr3:uid="{FA10D21D-A046-4812-AAF1-EE94BD98A442}" name="Name" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{4B62B6A5-AB9B-4B0A-B677-06970FE3B05C}" name="How to demo" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{9CB84775-431F-46EB-AF1A-30208D3E0DDB}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{45651187-7C4C-426E-8BC7-943CD802C12A}" name="#" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{FA10D21D-A046-4812-AAF1-EE94BD98A442}" name="Name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{4B62B6A5-AB9B-4B0A-B677-06970FE3B05C}" name="How to demo" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{9CB84775-431F-46EB-AF1A-30208D3E0DDB}" name="Notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -643,24 +657,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -677,372 +691,372 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>9</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A14" s="1">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>13</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>14</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>15</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+    </row>
+    <row r="20" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A20" s="1">
+        <v>16</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="6"/>
+    </row>
+    <row r="22" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>18</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>19</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>20</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="1"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>21</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>22</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>23</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="6"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>24</v>
+      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="1"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>25</v>
+      </c>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>26</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>27</v>
+      </c>
+      <c r="B31" s="1"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
         <v>28</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>8</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
-        <v>9</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A14" s="2">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
-        <v>11</v>
-      </c>
-      <c r="B15" s="2" t="s">
+      <c r="B32" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>29</v>
+      </c>
+      <c r="B33" s="1"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="1"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
         <v>30</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="B34" s="1"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
         <v>31</v>
       </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
-        <v>12</v>
-      </c>
-      <c r="B16" s="2" t="s">
+      <c r="B35" s="1"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="1"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
         <v>32</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
         <v>33</v>
       </c>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
-        <v>13</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
-        <v>14</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
-        <v>15</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A20" s="2">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
-        <v>17</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
-        <v>18</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="2">
-        <v>19</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
-        <v>20</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="2"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="2">
-        <v>21</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>22</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
-        <v>23</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="2">
-        <v>24</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="2">
-        <v>25</v>
-      </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>26</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="2">
-        <v>27</v>
-      </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A32" s="2">
+      <c r="B37" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="2">
-        <v>29</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="2">
-        <v>30</v>
-      </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
-        <v>31</v>
-      </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="2">
-        <v>32</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="2">
-        <v>33</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
initialisation of bsa Popup
</commit_message>
<xml_diff>
--- a/ProductBacklog.xlsx
+++ b/ProductBacklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\IdeaProjects\TUe-tycoon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB69A3F-5359-4D72-B68D-D31F3F180F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F2306C-9DF5-4A95-BB2A-9E89D3ADDC00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A18C0AB4-C4B4-4CEE-A740-ABC1F7C2C92A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
   <si>
     <t>Product Backlog TU/e Tycoon</t>
   </si>
@@ -192,6 +192,12 @@
   </si>
   <si>
     <t>when save file is missing, create one</t>
+  </si>
+  <si>
+    <t>total knowledge earned stat</t>
+  </si>
+  <si>
+    <t>at the bsa report see the total knowledge you earned in the game</t>
   </si>
 </sst>
 </file>
@@ -1044,8 +1050,12 @@
       <c r="A36" s="1">
         <v>32</v>
       </c>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
+      <c r="B36" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>53</v>
+      </c>
       <c r="D36" s="1"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>